<commit_message>
sync from doc_parser 9678cce14d0efbb810e8c79493261a73657ad16e (docling→wheel)
</commit_message>
<xml_diff>
--- a/genon/preprocessor/sample_files/monimo/monimo_stock_insight_sample.xlsx
+++ b/genon/preprocessor/sample_files/monimo/monimo_stock_insight_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="증권_AI차트뷰" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,117 +413,956 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>jong_name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>등록번호</t>
+          <t>jong_code</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>게시물라인번호</t>
+          <t>regt_no</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>종목코드</t>
+          <t>ntc_objline</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>종목명</t>
+          <t>detail_desc</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>뉴스일자</t>
+          <t>news_date</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>세부내용</t>
+          <t>md_stck_itm_c</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>kosc_stck_itm_c</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>nat_c</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADAC-0001</t>
+          <t>테슬라</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R2026071601</t>
+          <t>NQQUSATSLA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>000660</t>
-        </is>
+          <t>4556</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>{"trading_strategy": "현재 종가 346.44는 20일선(334.68)과 60일선(369.71) 사이에 위치하며, 5일선(350.73)은 종가 아래에 있음.&lt;BR&gt;&lt;BR&gt;8월 13일 RSI는 50.1로 과매도 또는 과매수 구간에 해당하지 않음.&lt;BR&gt;&lt;BR&gt;8월 14일 MACD(6.41)와 Signal(6.54)은 골든크로스 이전 상태로, MACD 곡선이 Signal 곡선 아래에 있음.&lt;BR&gt;&lt;BR&gt;8월 17일 주가가 볼린저 밴드 중심선(334.68) 위에서 움직이고 있으나 상한선(362.27)까지는 여유 있음.&lt;BR&gt;&lt;BR&gt;8월 18일 거래량증감률이 최근 2거래일 연속 감소한 가운데 주가등락률도 -1.09%로 하락하여, 단기 과열 신호는 확인되지 않음.&lt;BR&gt;&lt;BR&gt;8월 21일 이동평균선 배열상 단기 이평선(5일)이 10일선(346.31)에 근접한 상태에서 하향 돌파 가능성이 존재함.&lt;BR&gt;&lt;BR&gt;8월 24일 단기 분할 매수 후 20일선 이탈 시 손절하는 대응이 유효한 구간임.", "candle_</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20260716</t>
+          <t>20260827</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>{"trading_strategy": "단기 분할 매수 후 20일선 이탈 시 손절", "candle_analysis": "일봉 기준 장대양봉 출현 후 3일 연속 음봉으로 조정 중", "price_pattern_desc": "상승 삼각수렴 상단 돌파 시도 구간", "volume_change": "전일 대비 거래량 42% 증가", "technical_indicator_analysis": "RSI 61, MACD 골든크로스 유지", "overall_diagnosis": "관망 우위. 수급은 개선되었으나 단기 과열 신호가 함께 관측됨"}</t>
+          <t>US88160R1014</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TSLA.O</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADAC-0002</t>
+          <t>테슬라</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R2026071602</t>
+          <t>NQQUSATSLA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>005930</t>
-        </is>
+          <t>4556</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>analysis": {"summary": "8월 13일 양봉 이후 8월 14일 도지 형성으로 상승 힘 약화가 나타남.&lt;BR&gt;&lt;BR&gt;8월 17일 도지에서 저가 337.48, 8월 18일 양봉 저가 331.12로 저점 하락했으나 종가 336.87로 마감함.&lt;BR&gt;&lt;BR&gt;8월 19일 양봉(주가등락률 +4.23%)과 8월 21일 장대양봉(주가등락률 +5.14%, 거래량증감률 +95.02%)으로 상승 폭 확대됨.&lt;BR&gt;&lt;BR&gt;8월 24일 음봉(주가등락률 -3.83%)에서 종가 348.95로 20일선(330.13) 위 유지되며 조정 발생.&lt;BR&gt;&lt;BR&gt;8월 26일 연속 도지 형성으로 방향성 모호함이 지속되고 있음.", "potential_signal": "8월 21일 양봉 이후 8월 24일 음봉에서 거래량이 5857만 대비 3891만으로 감소 발생.&lt;BR&gt;&lt;BR&gt;8월 25일 음봉은 도지 캔들과 거래량 점진적 감소(2965만 → 2825만) 흐름을 동반함.&lt;BR&gt;&lt;BR&gt;8월 26일 추세 전환 신호는 확인되지 않음. 종가가 20일선 위에서 유지되고 있으나, 5일선 이하에서 마감 중임.&lt;BR&gt;&lt;BR&gt;8월 27일 주가 하락 시 20일선(334.68) 지지 여부 확인 필요."}, "price_pat</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>20260716</t>
+          <t>20260827</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>{"trading_strategy": "박스권 하단 접근 시 분할 매수", "candle_analysis": "5일 연속 도지형 캔들로 방향성 부재", "price_pattern_desc": "횡보 박스권 하단 지지 테스트", "volume_change": "전일 대비 거래량 8% 감소", "technical_indicator_analysis": "RSI 47, MACD 시그널선 하회", "overall_diagnosis": "중립. 거래량 동반 돌파 확인 후 대응이 유효"}</t>
+          <t>US88160R1014</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TSLA.O</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>테슬라</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NQQUSATSLA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4556</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tern_desc": "8월 13일 종가 339.96에서 상승해 8월 14일 342.27로 마감하며 주가등락률 +0.68% 기록함.&lt;BR&gt;&lt;BR&gt;8월 17일 339.30으로 소폭 하락한 후 8월 18일 336.87로 추가 하락했으나, 8월 19일 351.12로 급등하며 +4.23% 나타남.&lt;BR&gt;&lt;BR&gt;8월 20일 345.13으로 조정 후, 8월 21일 362.86으로 급등(+5.14%)하며 최근 고점 형성.&lt;BR&gt;&lt;BR&gt;8월 24일 348.95로 하락(-3.83%)하며 이전 상승분 일부 반납.&lt;BR&gt;&lt;BR&gt;8월 25일 350.25, 8월 26일 346.44로 소폭 등락하며 최근 상승 추세 후 조정 국면에 진입했습니다.", "volume</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>US88160R1014</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TSLA.O</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>테슬라</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NQQUSATSLA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4556</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>_change": "8월 13일 거래량 3408만에서 8월 14일 4515만으로 증가(거래량증감률 +32.47%)됨.&lt;BR&gt;&lt;BR&gt;8월 17일 2544만으로 감소, 8월 18일 2781만, 8월 19일 3627만으로 증가세로 전환됨.&lt;BR&gt;&lt;BR&gt;8월 20일 3003만으로 감소했으나, 8월 21일 5857만으로 급증(거래량증감률 +95.02%)하며 상승장에 동반된 거래량 확대 발생.&lt;BR&gt;&lt;BR&gt;8월 24일 3891만, 8월 25일 2965만, 8월 26일 2825만으로 거래량이 점진적으로 감소 중임.", "technical_indicator_analysis": {"RSI": "8월 13일 RSI 47.72에서 8월 14일 48.82로 상승함.&lt;BR&gt;&lt;BR&gt;8월 17일 47.44, 8월 18일 46.28로 하락했으나, 8월 19일 53.43으로 과매수 구간 진입 전 수준으로 반등.&lt;BR&gt;&lt;BR&gt;8월 21일 58.0까지 상승했으나, 이후 8월 24일 51.35, 8월 25일 51.91, 8월 26일 50.1로 점진적 하락 중.&lt;BR&gt;&lt;BR&gt;8월 27일 RSI는 30 이하 또는 70 이상 구간에 없으며, 과매도·과매수 신호는 발생하지 않음.", "MA</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>US88160R1014</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TSLA.O</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>테슬라</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NQQUSATSLA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4556</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CD": "8월 13일 MACD 4.17에서 8월 14일 5.35로 증가하며 상승 모멘텀 강화됨.&lt;BR&gt;&lt;BR&gt;8월 17일 6.20, 8월 18일 6.35로 정점 부근에 도달한 후, 8월 19일 6.09로 하락 전환.&lt;BR&gt;&lt;BR&gt;8월 20일 6.90으로 반등했으나, 8월 21일 6.72로 다시 하락하며 추세 둔화됨.&lt;BR&gt;&lt;BR&gt;8월 24일 7.79로 급등했으나, 8월 25일 7.05, 8월 26일 6.41로 하락하며 조정 중.&lt;BR&gt;&lt;BR&gt;8월 27일 MACD 곡선은 Signal 곡선을 8월 20일 이후 지속적으로 상회했으나, 최근 간격이 좁혀지고 있음.", "SUBtotal": "RSI는 50 부근에서 등락하며 중립 구간 유지 중이며, MACD는 여전히 Signal 위에 있으나 상승 폭 둔화됨.&lt;BR&gt;&lt;BR&gt;이동평균선은 5일선(350.73)이 10일선(346.31)에 근접한 상태에서 종가가 하향 밀집됨.&lt;BR&gt;&lt;BR&gt;볼린저 밴드는 중심선(334.68) 위에서 주가 움직임이 지속되고 있으나, 상한선(362.27)까지는 여유 있음.&lt;BR&gt;&lt;BR&gt;MACD와 RSI 모두 명확한 반전 신호는 나타나지 않았으며, 단기 조정 국면으로 해석 가능함."}, "overall_</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>US88160R1014</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TSLA.O</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>테슬라</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NQQUSATSLA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>4556</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>diagnosis": "최근 주가는 장대양봉 이후 음봉과 연속 도지 캔들이 나타나며 단기 조정 국면에 진입했습니다.&lt;BR&gt;&lt;BR&gt;거래량은 상승장에서 급증했다가 점차 감소하는 흐름을 보이고 있으며, &lt;strong&gt;종가가 5일 이평선 아래에서 지속 마감되면서 단기 상승 모멘텀이 약화되고 있습니다.&lt;/strong&gt;&lt;BR&gt;&lt;BR&gt;보조지표상 RSI는 중립 구간을 유지하고 있고 MACD도 시그널 상회 상태이나, 두 지표 모두 상승 폭이 둔화되며 추가적인 방향성 결정을 위한 관찰이 필요합니다."}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>US88160R1014</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>TSLA.O</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"trading_strategy": "현재 종가 215.04는 20일선(215.83) 아래에 위치하며, 5일선(213.63)은 10일선(218.09) 하향 돌파 후 하락 추세에 있습니다.&lt;BR&gt;&lt;BR&gt;8월 13일 MACD(-1.58)가 Signal선(0.72) 아래에 위치하고, 0선 하향 돌파로 중기 하락 추세 전환 신호를 나타냅니다.&lt;BR&gt;&lt;BR&gt;8월 14일 RSI(51.64)는 과매도 구간(30 이하)이나 과매수 구간(70 이상)에 있지 않으며, 최근 하락 추세와 함께 감소 흐름입니다.&lt;BR&gt;&lt;BR&gt;8월 17일 볼린저밴드 기준, 현재 주가는 중심선(215.83) 근접 위치에서 상한선(231.73)과 하한선(199.93) 사이에서 중립 구간에 머물고 있습니다.&lt;BR&gt;&lt;BR&gt;8월 18일 거래량은 8월 24일에 증가율 +34.30%로 확대된 후, 8월 26일 기준 전일 대비 +24.79% 증가한 상태로 하락장에서 거래량 확대가 지속되고 있습니다.&lt;BR&gt;&lt;BR&gt;8월 21일 박스권 하단 접근 시 분할 매수하되 20일선 회복 실패 시 비중 축소가 유효합니다.", "candle_</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>analysis": {"summary": "8월 13일부터 19일까지 종가 기준 등락이 반복되며 도지형 캔들이 3회 발생하여 시장의 관성 상태를 나타냅니다.&lt;BR&gt;&lt;BR&gt;8월 18일 음봉 이후 8월 19일 음봉이 이어졌고, 8월 20일부터 21일까지 연속 음봉 발생으로 하락 흐름이 강화됩니다.&lt;BR&gt;&lt;BR&gt;8월 24일 음봉(-2.91%)에서 거래량이 전일 대비 +34.30% 증가하며 매도 압력이 두드러지게 나타납니다.&lt;BR&gt;&lt;BR&gt;8월 26일은 양봉이 발생했으나, 종가는 여전히 20일선 아래에 머무르고 있어 반등보다는 일시적 회복으로 해석됩니다.", "potentia</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>l_signal": "8월 24일 음봉에서 거래량 증가와 함께 주가 하락이 나타나 매도 신호로 작용할 수 있습니다.&lt;BR&gt;&lt;BR&gt;8월 25일 최근 2영업일 연속 양봉이 발생했으나 20일선 재돌파 실패와 MACD 하락 지속으로 상승 신뢰도가 낮습니다.&lt;BR&gt;&lt;BR&gt;8월 26일 향후 20일선(215.83) 상향 돌파와 거래량 감소 시 조정 종료 신호로 해석될 수 있으며, 현재는 관망 기조가 적절합니다."}, "price_pattern_desc": "8월 13일 종가 225.30에서 소폭 상승 후, 8월 14일부터 18일까지 종가는 219.74로 하락하며 등락을 반복합니다.&lt;BR&gt;&lt;BR&gt;8월 19일부터 21일까지 3영업일 연속 음봉 발생하며 주가등락률 -0.99%, -0.33%, -0.98%로 하락 흐름이 이어집니다.&lt;BR&gt;&lt;BR&gt;8월 24일 주가등락률 -2.91%로 급락하며 저점 재하향 흐름을 나타냅니다.&lt;BR&gt;&lt;BR&gt;8월 25일과 26일 각각 +2.19%, +0.93% 반등했으나, 여전히 8월 13일 대비 종가 수준은 낮은 상태입니다.", "volume</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>_change": "8월 13일 거래량 98,072,310에서 8월 14일 75,311,153으로 -23.21% 감소하며 거래 위축이 발생합니다.&lt;BR&gt;&lt;BR&gt;8월 17일부터 18일로 넘어가며 거래량이 +12.76% 증가하고, 8월 19일에는 -6.67% 감소합니다.&lt;BR&gt;&lt;BR&gt;8월 24일 거래량이 전일 대비 +34.30% 급증하며 주가 하락과 동반된 매도 물량 증가가 확인됩니다.&lt;BR&gt;&lt;BR&gt;8월 25일에는 -9.63% 감소했으나 8월 26일 다시 +24.79% 증가하며 하락장에서 변동성 확대가 지속됩니다.", "technical_indi</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>cator_analysis": {"RSI": "RSI는 8월 13일 63.19에서 점차 하락하여 8월 24일 44.65까지 감소하여 과매수 영역에서 벗어납니다.&lt;BR&gt;&lt;BR&gt;8월 26일 기준 RSI는 51.64로 중립 구간에 위치하며, 주가 반등에도 불구하고 상승 모멘텀은 약합니다.&lt;BR&gt;&lt;BR&gt;8월 26일 주가 하락과 RSI 하락이 동반되어 일반 하락 다이버전스는 발생하지 않으며, 추세 동행 상태입니다.", "MACD": "MACD는 8월 13일 2.69에서 점차 감소하여 8월 19일 1.52, 8월 20일 0.74로 떨어지고, 8월 21일 0.11까지 하락합니다.&lt;BR&gt;&lt;BR&gt;8월 24일 MACD는 -0.50으로 0선 하향 돌파하며 중기 하락 추세 전환을 나타냅니다.&lt;BR&gt;&lt;BR&gt;8월 26일 MACD(-1.58)는 Signal선(0.72) 아래에서 확대되는 하락 폭을 보이며 추가 조정 가능성을 시사합니다.", "SUBt</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>otal": "MACD는 0선 하향 돌파와 Signal선 하향 크로스로 하락 추세 신호를 확정 지었고, RSI는 중립권에서 하향 추세를 유지합니다.&lt;BR&gt;&lt;BR&gt;이동평균선은 5일선이 10일선 및 20일선 아래에 위치하며 하락 정배열 구조입니다.&lt;BR&gt;&lt;BR&gt;볼린저밴드 중심선(215.83)이 저항선 역할을 하며, 현재 주가는 중심선 근처에서 반복적으로 등락하고 있습니다.&lt;BR&gt;&lt;BR&gt;거래량은 하락일에 증가하고 반등일에 감소하는 패턴으로, 매도 압력이 우세한 시장 구조입니다."}, "overall_</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>엔비디아</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NQQUSANVDA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>4558</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>diagnosis": "현재 주가는 20일선 아래에서 등락을 반복하며 하락 추세가 지속되고 있습니다.&lt;BR&gt;&lt;BR&gt;이동평균선 정배열과 MACD의 0선 하향 돌파가 중기 하락 전환을 시사합니다.&lt;BR&gt;&lt;BR&gt;&lt;strong&gt;8월 24일 급락장에서 거래량이 급증하며 매도 압력이 강화된 점&lt;/strong&gt;은 시장 심리가 위축되고 있음을 나타내고, 반등일에 거래량이 감소하는 등 상승 모멘텀이 취약합니다.&lt;BR&gt;&lt;BR&gt;RSI는 중립권에 위치하나 상승 폭이 제한적이며, 20일선 재상향 돌파와 거래량 축소가 확인되기 전까지는 조정 국면이 이어질 가능성이 높습니다."}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>US67066G1040</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NVDA.O</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>팔란티어 테크놀로지스</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NQQUSAPLTR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>4560</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>&lt;h3&gt;매매 전략&lt;/h3&gt;&lt;p&gt;현재 종가 177.27은 5일선(175.96)과 10일선(175.21)을 상회하며 단기 이동평균 대비 강세를 나타내고 있습니다. 20일선(164.67)은 종가 기준으로 지지선 역할을 하고 있으며, 주가가 볼린저 밴드 중심선(164.67) 위에서 거래되고 있습니다.&lt;/p&gt;&lt;h3&gt;일자별 지표&lt;/h3&gt;&lt;table&gt;&lt;tr&gt;&lt;th&gt;일자&lt;/th&gt;&lt;th&gt;종가&lt;/th&gt;&lt;th&gt;거래량&lt;/th&gt;&lt;th&gt;RSI&lt;/th&gt;&lt;th&gt;MACD&lt;/th&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 13일&lt;/td&gt;&lt;td&gt;179.01&lt;/td&gt;&lt;td&gt;36,178,448&lt;/td&gt;&lt;td&gt;72.89&lt;/td&gt;&lt;td&gt;6.13&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 14일&lt;/td&gt;&lt;td&gt;174.04&lt;/td&gt;&lt;td&gt;23,923,902&lt;/td&gt;&lt;td&gt;68.14&lt;/td&gt;&lt;td&gt;</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>US69608A1088</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PLTR.O</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>팔란티어 테크놀로지스</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NQQUSAPLTR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>4560</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>5.94&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 17일&lt;/td&gt;&lt;td&gt;172.55&lt;/td&gt;&lt;td&gt;24,416,714&lt;/td&gt;&lt;td&gt;66.73&lt;/td&gt;&lt;td&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 18일&lt;/td&gt;&lt;td&gt;171.54&lt;/td&gt;&lt;td&gt;27,954,443&lt;/td&gt;&lt;td&gt;65.74&lt;/td&gt;&lt;td&gt;3.98&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 19일&lt;/td&gt;&lt;td&gt;175.19&lt;/td&gt;&lt;td&gt;35,902,379&lt;/td&gt;&lt;td&gt;67.61&lt;/td&gt;&lt;td&gt;2.92&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 20일&lt;/td&gt;&lt;td&gt;173.96&lt;/td&gt;&lt;td&gt;26,756,975&lt;/td&gt;&lt;td&gt;66.30&lt;/td&gt;&lt;td&gt;2.29&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 21일&lt;/td&gt;&lt;td&gt;179.94&lt;/td&gt;&lt;td&gt;40,904,529&lt;/td&gt;&lt;td&gt;69.41&lt;/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>US69608A1088</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PLTR.O</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>팔란티어 테크놀로지스</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NQQUSAPLTR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4560</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">td&gt;&lt;td&gt;1.55&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 24일&lt;/td&gt;&lt;td&gt;175.89&lt;/td&gt;&lt;td&gt;84,667,386&lt;/td&gt;&lt;td&gt;64.52&lt;/td&gt;&lt;td&gt;1.37&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 25일&lt;/td&gt;&lt;td&gt;172.73&lt;/td&gt;&lt;td&gt;24,458,630&lt;/td&gt;&lt;td&gt;61.76&lt;/td&gt;&lt;td&gt;0.73&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;8월 26일&lt;/td&gt;&lt;td&gt;177.27&lt;/td&gt;&lt;td&gt;27,736,335&lt;/td&gt;&lt;td&gt;63.19&lt;/td&gt;&lt;td&gt;-0.09&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;h3&gt;거래량 변화&lt;/h3&gt;&lt;p&gt;8월 13일 거래량 36,178,448에서 8월 14일 23,923,902로 감소하며 주가 하락과 함께 거래량 감소가 나타났습니다. 8월 21일 40,904,529로 전일 대비 52.87% 증가하며 </t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>US69608A1088</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>PLTR.O</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>팔란티어 테크놀로지스</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NQQUSAPLTR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>4560</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>급등일과 동반된 증가세를 보였고, 8월 24일 84,667,386으로 급증했으나 8월 25일 24,458,630으로 감소했다가 8월 26일 27,736,335로 다시 증가했습니다.&lt;/p&gt;&lt;h3&gt;종합 진단&lt;/h3&gt;&lt;p&gt;최근 주가는 단기 이동평균선을 상회하며 강세 흐름을 유지하고 있으며, 볼린저 밴드 중심선 위에서 거래되어 상승 여력이 열려 있습니다. 그러나 &lt;strong&gt;MACD가 시그널선을 하향 돌파하며 매도 신호 유사한 상태로 전환&lt;/strong&gt;되었고, RSI 역시 주가 고점 대비 낮은 고점을 형성하며 일반 하락 다이버전스 유사 흐름을 보여 상승 모멘텀 약화가 의심됩니다. 8월 21일 양봉 재진입과 거래량 증가로 단기 반등 신호가 나타났으나, 주요 보조지표들의 불일치가 지속되고 있어 향후 추가적인 방향성 확인이 필요합니다.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>US69608A1088</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>PLTR.O</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>리게티 컴퓨팅</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NQQUSARGTI</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>현재 주가는 20일선(17.15) 아래에서 형성되며, 단기 이동평균(5일 16.68)이 장기 이동평균(10일 17.42)을 하향 돌파한 상태입니다. RSI는 45.76으로 과매도 구간 직전에 위치하며 과거 대비 낮은 수준에서 하락 추세입니다. MACD 값은 -0.06으로 Signal선(0.3)을 하향 돌파한 이후 음의 영역에서 확대되는 흐름입니다.
+볼린저 밴드 기준 현재 주가는 중심선(17.15) 아래에서 거래</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>US76655K1034</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>RGTI.O</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>리게티 컴퓨팅</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NQQUSARGTI</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>되며, 하한선(14.85)까지는 여유가 있습니다. 거래량은 8월 24일과 21일에 증가했으며, 8월 13일과 14일 연속 유성형 캔들과 양봉이 나타난 후 8월 17일 음봉이 형성되며 상승 흐름이 꺾였습니다.
+8월 18일에는 고가 대비 종가 하락 폭이 크고 윗꼬리가 긴 유성형 캔들이 발생하며 종일 고가를 상회하는 가격 탐색 후 되돌림이 나타났습니다. 8월 19일과 20일 연속 음봉이 이어졌고, 8월 21일 장대양</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>US76655K1034</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>RGTI.O</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>리게티 컴퓨팅</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>NQQUSARGTI</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>4566</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>봉이 발생하며 반등했으나 다음 날 다시 음봉으로 전환되었습니다.
+8월 24일 장대음봉 발생 후 8월 25일과 26일 소폭 반등과 하락이 반복되며 불확실성 있는 흐름이 지속되고 있습니다. 최근 유성형 캔들이 반복적으로 나타나고, 고점 인식 후 하락 반전 흐름이 반복되고 있어 단기 고점 인식 후 조정 국면으로 해석할 수 있습니다. 현재 캔들 패턴과 거래량 흐름은 상승 모멘텀 부족을 시사하며, 반등 지속력이 약합니다.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>20260827</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>US76655K1034</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>RGTI.O</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>US</t>
         </is>
       </c>
     </row>

</xml_diff>